<commit_message>
Segunda revisión de cierre: pausa sin trabajo, posición del sensor y documentación
- Pausar sin trabajo abierto (web o botonera) deja el telar apagado, no pausado.
- Reporte del sensor: repeticion_en_fila solo válida junto a una fila válida y dentro de sus repeticiones.
- Terminar trabajo, retroceder y cerrar sesión marcan la generación (no se vuelve a sumar al tejido).
- Documentos: código de recuperación fijo y cifrado, fuente en plaqueta aparte, capacitores de 100 nF,
  rutas de la API que faltaban en el README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Componentes_en_placa.xlsx
+++ b/documentacion_proyecto/Componentes_en_placa.xlsx
@@ -487,7 +487,7 @@
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>Las 2 patas AC a la red (sin polaridad) · +Vo y −Vo al bus de 5 V</t>
+          <t>Soldado en su propia plaqueta: bornera de 220 V a las 2 patas AC (sin polaridad) · +Vo y −Vo a la bornera de 5 V, que va a la placa principal</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
@@ -862,11 +862,11 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Soporte definitivo del circuito (reemplaza la protoboard)</t>
+          <t>Soporte definitivo del circuito (reemplaza la protoboard): la principal (ESP32, sensado y Bloques C y D), la de los módulos de relé y una chica para la fuente</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>La entrega final va soldada, no sobre protoboard.</t>
+          <t>La entrega final va soldada, no sobre protoboard. La fuente va aparte: lo que lleva 220 V queda separado de la baja tensión.</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Fijan la placa y los módulos al fondo del gabinete</t>
+          <t>Fijan las placas y los módulos de relé al fondo del gabinete</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Documentación: visita del 10/10 (prueba en protoboard, plaqueta en armado), componentes nuevos y funciones nuevas
- Registro de entrevistas y bitácora: reunión 7 del 10/10/2026; la conexión final pasa a ser la 8.
- Lista de componentes y componentes en placa: otra plaqueta y tiras de pines (19 de 2, 6 de 5, 4 de 6, 2 de 8).
- Manuales, estado del proyecto y documentación: una bobina por fila, Intercalar, hilado en la
  ficha y el PDF, estado del Nivel 2 (probado en protoboard, plaqueta en armado).
- Comentarios del esquema, el firmware y los README al día con la regla de una bobina por fila.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Componentes_en_placa.xlsx
+++ b/documentacion_proyecto/Componentes_en_placa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="6" min="1" max="1"/>
@@ -1070,11 +1070,11 @@
         </is>
       </c>
       <c r="C27" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Soporte definitivo del circuito (reemplaza la protoboard): la principal (ESP32, sensado y Bloques C y D), la de los módulos de relé y una chica para la fuente</t>
+          <t>Soporte definitivo del circuito (reemplaza la protoboard): la principal (ESP32, sensado y Bloques C y D), la de los módulos de relé y una chica para la fuente. Se suma una más (10/10/2026): con todo probado en protoboard, se está haciendo la plaqueta para probar todo de manera correcta</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
@@ -1197,6 +1197,34 @@
       <c r="F31" s="10" t="inlineStr">
         <is>
           <t>Etapa provisoria con cinta doble faz; el montaje definitivo va con separadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="7">
+      <c r="A32" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Tiras de pines (2x, 5x, 6x y 8x)</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Conectores enchufables en la plaqueta para el ESP32, los módulos y los cables</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>19 tiras de 2 pines · 6 de 5 · 4 de 6 · 2 de 8</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Se suman el 10/10/2026. Permiten sacar módulos y cables sin desoldar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Relés: conexión final en todos los documentos y resistencias de protección con margen
- Resistencia de protección: 220 Ω 2 W hasta 15 V y 470 Ω 3 W de 15 a 30 V
  (con un corto, a 15 V disipa 1,02 W y a 30 V 1,9 W: con 1 W y 2 W quedaba
  al límite). Diagramas regenerados.
- Conexionado del Nivel 2 (figura 2 nueva), Guía de los Bloques C y D y
  Estado del proyecto con la conexión final; las conexiones en paralelo o
  en serie con el lector quedan descartadas.
- Planillas de componentes: zócalo DIP-6, resistencia de protección,
  10 kΩ ½ W y borneras de 4 vías (precio a completar, los totales no
  cambian). Componentes en placa se imprime apaisada y sin texto cortado.
- config.h y la prueba de mesa del relé: comentarios al día (el firmware
  viene con PORCENTAJE_SELECCION en 0).
- Guía LCA110: 10 páginas, aclaración de la resistencia de 330 Ω.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Componentes_en_placa.xlsx
+++ b/documentacion_proyecto/Componentes_en_placa.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Componentes en placa" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Componentes en placa'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
@@ -125,7 +127,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -159,6 +161,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -411,9 +416,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="6" min="1" max="1"/>
@@ -458,7 +463,7 @@
     </row>
     <row r="2" ht="15" customHeight="1" s="7">
       <c r="A2" s="9" t="n"/>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>── ETAPA 1 · ALIMENTACIÓN (220 V) ──</t>
         </is>
@@ -468,7 +473,7 @@
       <c r="E2" s="9" t="n"/>
       <c r="F2" s="9" t="n"/>
     </row>
-    <row r="3" ht="21.75" customHeight="1" s="7">
+    <row r="3" ht="37.5" customHeight="1" s="7">
       <c r="A3" s="10" t="n">
         <v>1</v>
       </c>
@@ -554,7 +559,7 @@
     </row>
     <row r="6" ht="15" customHeight="1" s="7">
       <c r="A6" s="9" t="n"/>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>── ETAPA 2 · CONTROL (salidas a la botonera) ──</t>
         </is>
@@ -650,7 +655,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" s="7">
       <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>── ETAPA 3 · SENSADO (lectura de la botonera) ──</t>
         </is>
@@ -660,7 +665,7 @@
       <c r="E10" s="9" t="n"/>
       <c r="F10" s="9" t="n"/>
     </row>
-    <row r="11" ht="15" customHeight="1" s="7">
+    <row r="11" ht="26" customHeight="1" s="7">
       <c r="A11" s="10" t="n">
         <v>7</v>
       </c>
@@ -688,7 +693,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="7">
+    <row r="12" ht="26" customHeight="1" s="7">
       <c r="A12" s="10" t="n">
         <v>8</v>
       </c>
@@ -716,7 +721,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="63.75" customHeight="1" s="7">
+    <row r="13" ht="72" customHeight="1" s="7">
       <c r="A13" s="10" t="n">
         <v>9</v>
       </c>
@@ -744,7 +749,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="7">
+    <row r="14" ht="26" customHeight="1" s="7">
       <c r="A14" s="10" t="n">
         <v>10</v>
       </c>
@@ -774,7 +779,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" s="7">
       <c r="A15" s="9" t="n"/>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>── COMPONENTES PASIVOS ──</t>
         </is>
@@ -840,7 +845,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" s="7">
+    <row r="18" ht="26" customHeight="1" s="7">
       <c r="A18" s="10" t="n">
         <v>13</v>
       </c>
@@ -870,7 +875,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" s="7">
       <c r="A19" s="9" t="n"/>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>── ETAPA 4 · NIVEL 2 (Bloques C y D: se suman a la placa principal al armarlos) ──</t>
         </is>
@@ -880,7 +885,7 @@
       <c r="E19" s="9" t="n"/>
       <c r="F19" s="9" t="n"/>
     </row>
-    <row r="20" ht="30" customHeight="1" s="7">
+    <row r="20" ht="26" customHeight="1" s="7">
       <c r="A20" s="10" t="n">
         <v>14</v>
       </c>
@@ -908,7 +913,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="7">
+    <row r="21" ht="26" customHeight="1" s="7">
       <c r="A21" s="10" t="n">
         <v>15</v>
       </c>
@@ -964,7 +969,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1" s="7">
+    <row r="23" ht="37.5" customHeight="1" s="7">
       <c r="A23" s="10" t="n">
         <v>17</v>
       </c>
@@ -978,21 +983,21 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Corta la señal de cada lector óptico (uno por bobina de selección)</t>
+          <t>Da la señal en lugar de cada lector óptico (uno por bobina de selección)</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>pin1←R 330 Ω←GPIO 18/19/21/22 · pin2→GND · pin4 y pin6 al lector (serie o paralelo) · pin3 y 5 sin conectar</t>
+          <t>pin1←R 330 Ω←GPIO 18/19/21/22 · pin2→GND · pin4←R de protección←+ del conector del lector · pin6→señal del lector · pin3 y 5 sin conectar</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>La salida (4 y 6) queda aislada del ESP32: nunca unir sus cables con el GND del ESP32.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="7">
+          <t>La salida (4 y 6) queda aislada del ESP32: nunca unir sus cables con el GND del ESP32. Conexión final: diagramas/hardware/conexion_final_rele.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1" s="7">
       <c r="A24" s="10" t="n">
         <v>18</v>
       </c>
@@ -1049,24 +1054,40 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="7">
-      <c r="A26" s="9" t="n"/>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>── MONTAJE Y CONEXIONADO ──</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="7">
+      <c r="A26" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Zócalo DIP de 6 patas</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Permite cambiar un LCA110 sin desoldar</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Soldado en la placa; el relé va enchufado</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>La muesca del zócalo y la del relé, del lado de la pata 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1" s="7">
       <c r="A27" s="10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Placa universal perforada</t>
+          <t>Resistencia de protección (220 Ω 2 W o 470 Ω 3 W)</t>
         </is>
       </c>
       <c r="C27" s="10" t="n">
@@ -1074,111 +1095,95 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Soporte definitivo del circuito (reemplaza la protoboard): la principal (ESP32, sensado y Bloques C y D), la de los módulos de relé y una chica para la fuente. Se suma una más (10/10/2026): con todo probado en protoboard, se está haciendo la plaqueta para probar todo de manera correcta</t>
+          <t>Lado del telar: limita la corriente si hay un error de cableado</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Entre el + del conector de cada lector y el pin 4 de su LCA110</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>La entrega final va soldada, no sobre protoboard. La fuente va aparte: lo que lleva 220 V queda separado de la baja tensión.</t>
+          <t>220 Ω 2 W si el lector se alimenta con hasta 15 V; 470 Ω 3 W de 15 a 30 V. Del lado del telar: nunca al GND del ESP32.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="7">
       <c r="A28" s="10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Gabinete IP65 + prensacables</t>
+          <t>Resistencia 10 kΩ 1/2 W (lado del telar)</t>
         </is>
       </c>
       <c r="C28" s="10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Protege el nodo del polvo y la pelusa textil</t>
+          <t>Deja la señal en 0 V (papel) con el relé abierto</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Entre la señal y el − del conector de cada lector</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>Montado en pared o columna, no sobre el chasis del telar.</t>
+          <t>Del lado del telar: nunca al GND del ESP32.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="7">
-      <c r="A29" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Borneras de tornillo</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>Conexión de los cables que entran y salen del gabinete</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>Red, bus de 5 V y los 3 pares del telar</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>Permiten desconectar sin desoldar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="53.25" customHeight="1" s="7">
+      <c r="A29" s="9" t="n"/>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>── MONTAJE Y CONEXIONADO ──</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="72" customHeight="1" s="7">
       <c r="A30" s="10" t="n">
         <v>23</v>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Cable multifilar 6 conductores, 1 mm²</t>
+          <t>Placa universal perforada</t>
         </is>
       </c>
       <c r="C30" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Lleva la señal de los 3 botones hasta el gabinete: el mismo par sirve para el relé y para el sensado</t>
+          <t>Soporte definitivo del circuito (reemplaza la protoboard): la principal (ESP32, sensado y Bloques C y D), la de los módulos de relé y una chica para la fuente. Se suma una más (10/10/2026): con todo probado en protoboard, se está haciendo la plaqueta para probar todo de manera correcta</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>Un par por botón, del telar a las borneras del gabinete</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>Sin blindaje. Se descartó el cable mallado tras consulta profesional: la señal de contacto seco a 24 V tiene inmunidad de sobra, el telar no tiene variador de frecuencia y su electrónica está en una caja metálica que contiene el ruido. Único recaudo: no correrlo pegado y en paralelo al cable del motor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="21.75" customHeight="1" s="7">
+          <t>La entrega final va soldada, no sobre protoboard. La fuente va aparte: lo que lleva 220 V queda separado de la baja tensión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="7">
       <c r="A31" s="10" t="n">
         <v>24</v>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Separadores / standoffs + tornillos</t>
+          <t>Gabinete IP65 + prensacables</t>
         </is>
       </c>
       <c r="C31" s="10" t="n">
@@ -1186,7 +1191,7 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Fijan las placas y los módulos de relé al fondo del gabinete</t>
+          <t>Protege el nodo del polvo y la pelusa textil</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -1196,33 +1201,117 @@
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>Etapa provisoria con cinta doble faz; el montaje definitivo va con separadores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="7">
+          <t>Montado en pared o columna, no sobre el chasis del telar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="37.5" customHeight="1" s="7">
       <c r="A32" s="10" t="n">
         <v>25</v>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
+          <t>Borneras de tornillo</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Conexión de los cables que entran y salen del gabinete</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Red, bus de 5 V y los 3 pares del telar</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Permiten desconectar sin desoldar. El Bloque D suma 8 borneras de 4 vías en el lado del telar (dos por canal, en el conector del lector).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="60.5" customHeight="1" s="7">
+      <c r="A33" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Cable multifilar 6 conductores, 1 mm²</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Lleva la señal de los 3 botones hasta el gabinete: el mismo par sirve para el relé y para el sensado</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>Un par por botón, del telar a las borneras del gabinete</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Sin blindaje. Se descartó el cable mallado tras consulta profesional: la señal de contacto seco a 24 V tiene inmunidad de sobra, el telar no tiene variador de frecuencia y su electrónica está en una caja metálica que contiene el ruido. Único recaudo: no correrlo pegado y en paralelo al cable del motor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1" s="7">
+      <c r="A34" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Separadores / standoffs + tornillos</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Fijan las placas y los módulos de relé al fondo del gabinete</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>Etapa provisoria con cinta doble faz; el montaje definitivo va con separadores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1" s="7">
+      <c r="A35" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
           <t>Tiras de pines (2x, 5x, 6x y 8x)</t>
         </is>
       </c>
-      <c r="C32" s="10" t="n">
+      <c r="C35" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>Conectores enchufables en la plaqueta para el ESP32, los módulos y los cables</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>19 tiras de 2 pines · 6 de 5 · 4 de 6 · 2 de 8</t>
         </is>
       </c>
-      <c r="F32" s="10" t="inlineStr">
+      <c r="F35" s="10" t="inlineStr">
         <is>
           <t>Se suman el 10/10/2026. Permiten sacar módulos y cables sin desoldar.</t>
         </is>
@@ -1231,6 +1320,6 @@
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Plaqueta de sensado aparte, unida a la principal por J4
La guía paso a paso (md y Word), el diagrama de plaquetas, el índice, el README de diagramas, la
Guía del Bloque A y Componentes en placa describen ahora cinco plaquetas: la de sensado de la
botonera va aparte, con J4 (3,3 V, GND y GPIO 32, 33 y 34) y B1 doble por botón (un par de la
botonera y otro hacia NO y COM de su relé).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Componentes_en_placa.xlsx
+++ b/documentacion_proyecto/Componentes_en_placa.xlsx
@@ -1149,7 +1149,7 @@
       <c r="E29" s="9" t="n"/>
       <c r="F29" s="9" t="n"/>
     </row>
-    <row r="30" ht="72" customHeight="1" s="7">
+    <row r="30" ht="88" customHeight="1" s="7">
       <c r="A30" s="10" t="n">
         <v>23</v>
       </c>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Soporte definitivo del circuito (reemplaza la protoboard): la principal (ESP32, sensado y Bloques C y D), la de los módulos de relé y una chica para la fuente. Se suma una más (10/10/2026): con todo probado en protoboard, se está haciendo la plaqueta para probar todo de manera correcta</t>
+          <t>Soporte definitivo del circuito (reemplaza la protoboard): la principal (ESP32 y Bloques C y D), la de los módulos de relé y una chica para la fuente. Se suma una más (10/10/2026): con todo probado en protoboard, se está haciendo la plaqueta para probar todo de manera correcta. El sensado de la botonera va en su propia plaqueta impresa (diseñada en Proteus), unida a la principal por J4</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -1205,7 +1205,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="37.5" customHeight="1" s="7">
+    <row r="32" ht="40" customHeight="1" s="7">
       <c r="A32" s="10" t="n">
         <v>25</v>
       </c>
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="C32" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Red, bus de 5 V y los 3 pares del telar</t>
+          <t>Red, bus de 5 V y B1 en la plaqueta de sensado: dos por botón (el par de la botonera y el par que va a NO y COM de su relé)</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Gantt con las dos funciones (643 h) y la prueba del 17/10 en el telar
Tres tareas nuevas en la Etapa 07, cargadas en la planilla del Drive (7,12 a
7,14), y las fechas reales de 7,4 a 7,6. Con 643 horas el presupuesto pasa a
$40.095.441 (costo $32.076.353, ganancia $8.019.088): Estimación,
Modalidad, Documentación de Proyecto, sitio y figuras 11 y 13.

La prueba del 17/10/2026, en protoboard: el lector se alimenta con 15 a
30 V (resistencia de protección de 470 Ω 3 W), el sensor de pasada quedó
conectado y calibrado, y el primer canal seleccionó bien. Se registra en la
Bitácora, el Estado completo, la Documentación, las guías, las planillas,
los manuales y los Markdown.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Componentes_en_placa.xlsx
+++ b/documentacion_proyecto/Componentes_en_placa.xlsx
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Resistencia de protección (220 Ω 2 W o 470 Ω 3 W)</t>
+          <t>Resistencia de protección 470 Ω 3 W</t>
         </is>
       </c>
       <c r="C27" s="10" t="n">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>220 Ω 2 W si el lector se alimenta con hasta 15 V; 470 Ω 3 W de 15 a 30 V. Del lado del telar: nunca al GND del ESP32.</t>
+          <t>De 470 Ω 3 W porque el lector del C 201 se alimenta con 15 a 30 V (medido el 17/10/2026); con hasta 15 V sería de 220 Ω 2 W. Del lado del telar: nunca al GND del ESP32.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Documentación: pull-up interna en GPIO 32 y 33 del sensado
Los Word (con sus PDF), las planillas, los diagramas, los Markdown del firmware y la
verificación dicen lo mismo que el firmware: el 32 y el 33 usan la pull-up interna del
ESP32 y solo el 34 lleva su 10 kΩ. Las 6 resistencias compradas quedan 4 en uso y 2 de
repuesto, sin cambio de costos. Entrada del 21/10 en la Bitácora.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Componentes_en_placa.xlsx
+++ b/documentacion_proyecto/Componentes_en_placa.xlsx
@@ -808,7 +808,7 @@
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
@@ -817,12 +817,12 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>3 en los relés + 3 en el sensado</t>
+          <t>3 en los relés + 1 en el sensado (GPIO 34)</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>5 van a 3V3 y la de GPIO 27 va a GND (módulo activo-alto).</t>
+          <t>3 van a 3V3 (GPIO 25, 26 y 34) y la de GPIO 27 va a GND (módulo activo-alto). GPIO 32 y 33 usan la pull-up interna del ESP32.</t>
         </is>
       </c>
     </row>

</xml_diff>